<commit_message>
Vika 1: lokaskjal með nýjum heimilisföngum auglýsenda og Póstdreifingarblaði
Fyrirtækjablað uppfært úr svörum 01.10: KORA fær eintak líka á Seinakur 8,
Steindi/Heit gólf á Kópavogsbraut 88 í stað Turnahvarfs 4. Nýtt blað fyrir
Póstdreifingu (nafn, heimilisfang, póstnúmer, hverfanúmer) með 150 heimilum
og 9 eintökum auglýsenda, auk samantektar. Listinn var endurkeyrður með
nýjustu kaupskrá og er óbreyttur.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fts7wXaAbvyJ2CRF93qGGq
</commit_message>
<xml_diff>
--- a/svif_utsending_150.xlsx
+++ b/svif_utsending_150.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Fyrirtæki í bæklingi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Vika 1 (150)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Póstdreifing vika 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Samantekt" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,10 +62,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,383 +442,434 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fyrirtæki</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Síður</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tengiliður / netfang</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Heimilisfang (sendum eintak)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Eintak af bæklingi sent á</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Kennitala (reikningur)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Verð 1. mánuður án vsk</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Staða tölvupósts 01.10</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Heimild / athugasemd</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>VÍS tryggingar hf</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 3)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Trausti S. Hilmisson – traustih@vis.is</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Ármúla 3, 108 Reykjavík</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>690689-2009 (úr vefleit, staðfesta)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>30.000 kr.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Tilboð 24.08: 25.000 kr fyrsta mánuð – Trausti samþykkti | Verð skv. Helga 01.10</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 13:08 – ekkert svar enn</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tilboð 24.08: 25.000 kr fyrsta mánuð – Trausti samþykkti | Verð 30.000 skv. Helga 01.10</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>HK Lagnir ehf</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 4)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Hjörvar – hklagnir@hklagnir.is, 776-9319</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Flúðaseli 67, 109 Reykjavík (lögheimili skv. fyrirtækjaskrá)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>570122-0530 (af auglýsingunni)</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>25.000 kr.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 13:08 – ekkert svar enn</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>"Val í bækling hjá Svif" 17.08: 25.000 kr</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>REKK Import ehf (MAUS)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2 (bls. 5–6)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>rekk@rekk.is, 780 2200 / 847 2389</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Kristján – kristjan@webpro.is; rekk@rekk.is, 780 2200</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Katrínartúni 4, 105 Reykjavík</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>601117-0610 (rekk.is skilmálar + fyrirtækjaskrá)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>40.000 kr. (2 síður)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 13:09 á kristjan@webpro.is – ekkert svar enn</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Engin tölvupóstsamskipti fundust við REKK/MAUS – líklega samið símleiðis | Verð skv. Helga 01.10</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Gardínur.is</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 7)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Valdimar – valdimar@gardinur.is / sala@gardinur.is, 519-6886</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Dalbrekka 56, 200 Kópavogur</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>VANTAR – Gardinur ehf. skv. vefsíðu, finnst ekki undir því nafni í fyrirtækjaskrá</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>25.000 kr.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Líklega sama 25.000 kr tilboð og aðrir, en staðfesta | Verð skv. Helga 01.10</t>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 10:34 – ekkert svar enn</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Staðfesta kennitölu þegar Valdimar svarar | Verð skv. Helga 01.10</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>KORA ehf</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 8)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Kjartan Freyr – kjartan@kora.is (cc kristjan@webpro.is), 416-7777</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Katrínartún 4, 105 Reykjavík</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Kjartan Freyr Kjartansson – kjartan@kora.is, 847-2389 (cc kristjan@webpro.is)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Katrínartún 4, 105 Reykjavík  OG  Seinakur 8, 210 Garðabær (nýtt, skv. Kjartani 01.10)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>580918-0850 (úr pósti Kjartans)</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>25.000 kr.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 13:08 – SVAR 13:10: „Mátt alveg líka senda á Seinakur 8“ → tvö eintök</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>"fyrsta útgáfa Svifs" 17.08: 25.000 kr</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Stíflu- og myndavélaþjónustan ehf (Stíflan)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 9)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>stiflan@stiflan.is, 860-0938</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Ármúla 21, 108 Reykjavík</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>690307-0570 (af auglýsingunni)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>25.000 kr.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 13:07 – ekkert svar enn</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>"Bæklingur" 20.08: 25.000 kr</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>MJ Lausnir ehf</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 10)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>í gegnum Birta Media: birta@birtamedia.is / audur@birtamedia.is; mjlausnir.is 775-9931</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Hafnargata 35, 230 Reykjanesbær (mjlausnir.is)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>660620-0870 (hlekkur frá Birta Media)</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>25.000 kr.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 13:07 á Birta Media – ekkert svar enn</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Birta Media 20.08: "MJ Lausnir er til í að prufa þetta" eftir 25.000 kr tilboð</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Steindi ehf</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>2 (bls. 11–12)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Þór Þorsteinsson – thor@heitgolf.is; steindi@steindi.is, 430 8300</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Turnahvarf 4, 203 Kópavogur</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Kópavogsbraut 88, 200 Kópavogur (nýtt, skv. Þór 01.10 – í stað Turnahvarfs 4)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>700414-0350 (steindi.is)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>sjá Heit Gólf – 60.000 kr. samtals fyrir 3 síður (Steindi + Heit Gólf)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Mögulega 30.000 kr skv. þér – staðfesta | Verð skv. Helga 01.10</t>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>60.000 kr. samtals fyrir 3 síður (Steindi + Heit Gólf)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Sent 01.10 kl. 10:33 – SVAR 12:35: „Mátt senda hann á Kópavogsbraut 88, 200 Kópavogur“ + 12:36: vill PDF af bæklingnum á thor@heitgolf.is</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Verð skv. Helga 01.10 | Senda PDF á Þór</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Heitum Gólfum ehf (Heit Gólf)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>1 (bls. 13)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Þór Þorsteinsson – thor@heitgolf.is; heitgolf@heitgolf.is, 430 8300</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Turnahvarf 4, 203 Kópavogur</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Kópavogsbraut 88, 200 Kópavogur (nýtt, skv. Þór 01.10 – í stað Turnahvarfs 4)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>450207-1600 (heitgolf.is)</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>60.000 kr. samtals fyrir 3 síður (Steindi + Heit Gólf)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Sama svar og Steindi (einn tengiliður, Þór) – eitt eintak á Kópavogsbraut 88</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>"Val í svif" 17.08: 25.000 kr | Verð skv. Helga 01.10</t>
         </is>
@@ -841,92 +910,92 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nafn</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Heimilisfang</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Póstnúmer</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Staður</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Íbúð</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Einkunn</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Stig</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tegund</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Byggt</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Herb.</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Kaupsamningur</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Áætluð afhending</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Dagar frá afhendingu</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Afhendingarregla</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Fastanúmer</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Ástæða einkunnar</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Athugasemd</t>
         </is>
@@ -11851,6 +11920,3928 @@
         </is>
       </c>
       <c r="R151" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F160"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nafn</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Heimilisfang</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Póstnúmer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Staður</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Hverfanúmer (Póstdreifing)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Athugasemd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bergþórugata 7</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>101</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bragagata 33</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>101</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Grettisgata 46, íbúð 0302</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>101</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>íbúð 0302</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Leifsgata 18, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>101</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bauganes 3</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>102</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Reykjavíkurvegur 23</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>102</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hvassaleiti 103</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>103</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Drekavogur 14</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>104</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Efstasund 64</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>104</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kambsvegur 11</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>104</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kleppsvegur 94</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>104</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Skipasund 77</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>104</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Barmahlíð 23, íbúð 0201</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>105</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>íbúð 0201</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Birkihlíð 42, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>105</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bólstaðarhlíð 48, íbúð 0201</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>105</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>íbúð 0201</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bólstaðarhlíð 5, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>105</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Laugarnesvegur 112, íbúð 0105</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>105</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>íbúð 0105</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mávahlíð 11, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>105</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Otrateigur 18</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>105</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Rauðalækur 51, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>105</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Skipholt 24, íbúð 0201</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>105</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>íbúð 0201</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Stigahlíð 4, íbúð 0402</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>105</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>íbúð 0402</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ásholt 28</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>105</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Hagamelur 48, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>107</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Tómasarhagi 36, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>107</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Víðimelur 30, íbúð 0201</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>107</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>íbúð 0201</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Heiðargerði 3</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>108</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Heiðargerði 33</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>108</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Heiðargerði 43</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>108</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Háaleitisbraut 93</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>108</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Kúrland 26</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>108</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ljósaland 3</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>108</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Álftamýri 36, íbúð 0203</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>108</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>íbúð 0203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Ásgarður 123</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>108</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bakkasel 25</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>109</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Engjasel 66</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>109</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Engjasel 82</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>109</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Eyjabakki 7, íbúð 0202</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>109</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>íbúð 0202</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Ferjubakki 2, íbúð 0202</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>109</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>íbúð 0202</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Látrasel 12</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>109</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Seljabraut 46</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>109</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Strýtusel 10</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>109</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Strýtusel 13</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>109</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Stuðlasel 6</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>109</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Víkurbakki 8</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>109</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Eyktarás 15</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>110</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Hraunbær 158, íbúð 0301</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>110</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>íbúð 0301</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Seiðakvísl 5</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>110</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Þykkvibær 4</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>110</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Hamraberg 30</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>111</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Keilufell 4</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>111</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Torfufell 16</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>111</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Vesturberg 120, íbúð 0203</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>111</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>íbúð 0203</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Vesturberg 97</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>111</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Æsufell 6, íbúð 0706</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>111</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>íbúð 0706</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Fannafold 4</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>112</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Funafold 12</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>112</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Þorláksgeisli 46</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>113</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Vindheimar</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>162</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Lindarbraut 17</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>170</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Lindarbraut 24</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>170</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Melabraut 48</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>170</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Nesbali 20</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>170</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Nesbali 25</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>170</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sefgarðar 20</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>170</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Sefgarðar 28</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>170</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sævargarðar 7</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>170</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Seltjarnarnes</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Brekkugata 19</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>190</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Vogar</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Heiðargerði 16</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>190</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Vogar</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Vogagerði 17</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>190</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Vogar</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bræðratunga 24</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>200</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Daltún 17</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>200</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Fagrabrekka 25, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>200</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Fagrihjalli 10</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>200</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Hlíðarvegur 6</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>200</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Hlíðarvegur 61</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>200</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Kjarrhólmi 6, íbúð 0302</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>200</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>íbúð 0302</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Kópavogsbraut 63</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>200</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Lyngbrekka 23</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>200</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Þinghólsbraut 8</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>200</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Aratún 28</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>210</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bæjargil 110</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>210</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Efstilundur 8</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>210</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Faxatún 5</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>210</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Furulundur 2</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>210</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Hlíðarbyggð 3</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>210</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Hlíðarbyggð 33</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>210</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Hrísmóar 1, íbúð 0401</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>210</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>íbúð 0401</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Kjarrmóar 11</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>210</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Kjarrmóar 23</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>210</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Langafit 26</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>210</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Lindarflöt 40</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>210</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Markarflöt 9</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>210</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Móaflöt 12</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>210</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Naustahlein 26</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>210</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Smáraflöt 45</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>210</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Arnarhraun 9, íbúð 0201</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>220</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>íbúð 0201</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Brekkuhvammur 16</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>220</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Erluhraun 3</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>220</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Hellubraut 9</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>220</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Hjallabraut 70</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>220</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Kirkjuvegur 13</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>220</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Kirkjuvegur 3</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>220</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Klausturhvammur 30</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>220</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Langeyrarvegur 16</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>220</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Mávahraun 1</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>220</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Selvogsgata 20</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>220</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Smyrlahraun 19</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>220</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Smárahvammur 4</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>220</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Suðurgata 56</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>220</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Öldugata 26</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>220</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Ölduslóð 43</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>220</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Axlarás 39</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>221</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Glitvellir 14</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>221</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Hringhamar 8, íbúð 0202</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>221</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>íbúð 0202</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Stuðlaberg 48</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>221</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Hafnarfjörður</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Helguvík</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>225</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Garðabær (Álftanes)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Víðiholt 10</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>225</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Garðabær (Álftanes)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Faxabraut 31A</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>230</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Freyjuvellir 5</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>230</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Freyjuvellir 9</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>230</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Hafnargata 70</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>230</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Heiðarbraut 1E</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>230</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Heiðarvegur 21A</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>230</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Háaleiti 31</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>230</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Háteigur 20</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>230</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Suðurvellir 1</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>230</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Suðurvellir 7</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>230</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Sóltún 7, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>230</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Túngata 12, íbúð 0101</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>230</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>íbúð 0101</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Hlíðargata 32</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>245</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Suðurnesjabær</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Túngata 16</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>245</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Suðurnesjabær</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Bjarkartún 5</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>250</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Suðurnesjabær</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Háteigur 5</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>250</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Suðurnesjabær</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Skagabraut 13</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>250</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Suðurnesjabær</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Þórshamrar</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>250</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Suðurnesjabær</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Huldudalur 5</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>260</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Kirkjubraut 3</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>260</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Laufdalur 51</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>260</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Stapavellir 5</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>260</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Bogabraut 963A, íbúð 0204</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>262</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>íbúð 0204</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Skógarbraut 916C, íbúð 0106</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>262</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>íbúð 0106</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Skógarbraut 916C, íbúð 0207</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>262</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>íbúð 0207</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Arnartangi 23</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>270</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Krókabyggð 36</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>270</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Leirutangi 11A</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>270</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Leirutangi 22</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>270</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Leirvogstunga 12</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>270</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Litlagerði</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>270</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Til húseiganda</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Reykjavegur 86</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>270</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Mosfellsbær</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>VÍS tryggingar hf</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>Ármúli 3</t>
+        </is>
+      </c>
+      <c r="C152" s="4" t="n">
+        <v>108</v>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="inlineStr"/>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>HK Lagnir ehf (Hjörvar)</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>Flúðasel 67</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="inlineStr"/>
+      <c r="F153" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>REKK Import ehf (MAUS)</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Katrínartún 4</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr"/>
+      <c r="F154" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>Gardínur.is (Valdimar)</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Dalbrekka 56</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr"/>
+      <c r="F155" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>KORA ehf</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>Katrínartún 4</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr"/>
+      <c r="F156" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>Kjartan Freyr Kjartansson (KORA)</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Seinakur 8</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>Garðabær</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr"/>
+      <c r="F157" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda – nýtt heimilisfang skv. Kjartani 01.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>Stíflu- og myndavélaþjónustan ehf</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>Ármúli 21</t>
+        </is>
+      </c>
+      <c r="C158" s="4" t="n">
+        <v>108</v>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>Reykjavík</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="inlineStr"/>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>MJ Lausnir ehf</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Hafnargata 35</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="n">
+        <v>230</v>
+      </c>
+      <c r="D159" s="4" t="inlineStr">
+        <is>
+          <t>Reykjanesbær</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="inlineStr"/>
+      <c r="F159" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>Þór Þorsteinsson (Steindi / Heit gólf)</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Kópavogsbraut 88</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>Kópavogur</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr"/>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>Eintak auglýsanda – nýtt heimilisfang skv. Þór 01.10 (í stað Turnahvarfs 4)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>SVIF – vika 1</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Dreifing 3. október 2026 (Póstdreifing, límmiðamerking)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Listi búinn til</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1. október 2026 úr kaupskrá HMS með heimsent.py (miðað við áætlaðan afhendingardag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Heimili á lista</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Eintök til auglýsenda</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Samtals bæklingar</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Einkunn</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>A: 113, B: 37</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tegund</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Einbýli: 75, Sérbýli: 45, Fjölbýli: 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Fjölbýli með íbúðarnúmeri</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Dagar frá áætlaðri afhendingu</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>minnst 1, miðgildi 25, mest 81</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Afhendingarregla</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>notað: 144, ófullbúið (óviss): 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Kaupsamningar eftir mánuði</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2025-11: 1, 2025-12: 5, 2026-05: 29, 2026-06: 45, 2026-07: 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Eftir stað</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Reykjavík: 59, Hafnarfjörður: 20, Reykjanesbær: 19, Garðabær: 16, Kópavogur: 10, Seltjarnarnes: 8, Mosfellsbær: 7, Suðurnesjabær: 6, Vogar: 3, Garðabær (Álftanes): 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Reglur</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Notað húsnæði: afhending = kaupsamningur + 10 vikur. Selt ófullbúið: + 9 mánuðir (merkt óviss). Fullbúnar nýbyggingar, verktakakaup, ónothæfir samningar og atvinnuhúsnæði eru ekki á lista. Ekkert fer út fyrir áætlaðan afhendingardag og dettur út 150 dögum eftir hann.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Fjölbýli</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Íbúðarnúmer (hæð + íbúð) úr kaupskrá er á öllum fjölbýlisíbúðum, t.d. „Hraunbær 158, íbúð 0301“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Hverfanúmer</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Dálkurinn „Hverfanúmer“ á Póstdreifingarblaðinu er auður – Póstdreifing merkir hverfin sjálf. Heimilisföng utan dreifikerfis þeirra fara með Íslandspósti skv. verðskrá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Eftir að gera</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>1) Senda Póstdreifingarblaðið á Harald (haraldurb@postdreifing.is) í dag og gefa upp kennitölu fyrir dreifinguna. 2) Senda Þór (thor@heitgolf.is) PDF af bæklingnum. 3) Fá kennitölu Gardínur.is frá Valdimar. 4) Keyra heimsent.py run --commit þegar listinn er farinn.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>